<commit_message>
Fixed BOM and CPL file designators to avoid errors  on JLCPCB assembly page
</commit_message>
<xml_diff>
--- a/Gerbers/FreeRunner BOM.xlsx
+++ b/Gerbers/FreeRunner BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Armin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Austin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51AC0838-5FDD-4FDD-9BE6-62760AE018F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF5F2774-D83D-4250-9071-7BAC5F607FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{18CE6DBF-B421-447D-B0F0-1323BDBE6CB3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{18CE6DBF-B421-447D-B0F0-1323BDBE6CB3}"/>
   </bookViews>
   <sheets>
     <sheet name="FreeRunner Bapple Edition BOM" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="66">
   <si>
     <t>C1,C2,C3,C4</t>
   </si>
@@ -49,36 +49,18 @@
     <t>J2</t>
   </si>
   <si>
-    <t>Conn_01x06_Pin</t>
-  </si>
-  <si>
-    <t>1k</t>
-  </si>
-  <si>
     <t>R2,R3</t>
   </si>
   <si>
-    <t>10k</t>
-  </si>
-  <si>
     <t>R7</t>
   </si>
   <si>
-    <t>22k</t>
-  </si>
-  <si>
     <t>R8</t>
   </si>
   <si>
-    <t>5k</t>
-  </si>
-  <si>
     <t>R9</t>
   </si>
   <si>
-    <t>0 ohm</t>
-  </si>
-  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -109,9 +91,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Reference Designator</t>
-  </si>
-  <si>
     <t>Item #</t>
   </si>
   <si>
@@ -154,15 +133,9 @@
     <t>SMD</t>
   </si>
   <si>
-    <t>Green SMD LED</t>
-  </si>
-  <si>
     <t>KH-2.54PH-1X6P-L13.5-WT</t>
   </si>
   <si>
-    <t>48MHz Oscillator</t>
-  </si>
-  <si>
     <t>SCEYR48X0000018VRM</t>
   </si>
   <si>
@@ -199,9 +172,6 @@
     <t>FOJAN</t>
   </si>
   <si>
-    <t>R1, R4, R5, R6</t>
-  </si>
-  <si>
     <t>RC0402FR-0710KL</t>
   </si>
   <si>
@@ -214,9 +184,6 @@
     <t>Kinghelm</t>
   </si>
   <si>
-    <t>DBG0, DBG1, DBG2</t>
-  </si>
-  <si>
     <t>19-219/GHC-YR2T1B5Y/3T</t>
   </si>
   <si>
@@ -242,6 +209,15 @@
   </si>
   <si>
     <t>SMD,6.6x1.4mm</t>
+  </si>
+  <si>
+    <t>DBG0,DBG1,DBG2</t>
+  </si>
+  <si>
+    <t>R1,R4,R5,R6</t>
+  </si>
+  <si>
+    <t>Designator</t>
   </si>
 </sst>
 </file>
@@ -392,7 +368,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -581,6 +557,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -760,7 +742,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -782,6 +764,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="18" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1155,31 +1140,31 @@
   <sheetData>
     <row r="1" spans="1:15" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>36</v>
       </c>
       <c r="O1" s="1"/>
     </row>
@@ -1194,19 +1179,19 @@
         <v>4</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I2" s="5"/>
       <c r="N2" s="1"/>
@@ -1222,19 +1207,19 @@
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I3" s="5"/>
       <c r="N3" s="1"/>
@@ -1250,19 +1235,19 @@
         <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I4" s="5"/>
       <c r="N4" s="1"/>
@@ -1278,19 +1263,19 @@
         <v>4</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I5" s="5"/>
       <c r="N5" s="1"/>
@@ -1300,25 +1285,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C6" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I6" s="5"/>
       <c r="N6" s="1"/>
@@ -1334,19 +1319,19 @@
         <v>1</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I7" s="5"/>
       <c r="N7" s="1"/>
@@ -1356,25 +1341,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C8" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I8" s="5"/>
       <c r="N8" s="1"/>
@@ -1384,25 +1369,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C9" s="3">
         <v>2</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I9" s="5"/>
       <c r="N9" s="1"/>
@@ -1412,25 +1397,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C10" s="3">
         <v>1</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I10" s="5"/>
       <c r="N10" s="1"/>
@@ -1440,25 +1425,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3">
         <v>1</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I11" s="5"/>
       <c r="N11" s="1"/>
@@ -1468,25 +1453,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C12" s="3">
         <v>1</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I12" s="5"/>
       <c r="N12" s="1"/>
@@ -1496,25 +1481,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C13" s="3">
         <v>1</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I13" s="5"/>
       <c r="N13" s="1"/>
@@ -1524,25 +1509,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C14" s="3">
         <v>1</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I14" s="5"/>
       <c r="N14" s="1"/>
@@ -1552,25 +1537,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C15" s="3">
         <v>1</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I15" s="5"/>
       <c r="N15" s="1"/>
@@ -1580,25 +1565,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C16" s="3">
         <v>1</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I16" s="5"/>
       <c r="N16" s="1"/>
@@ -1608,25 +1593,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C17" s="3">
         <v>1</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I17" s="5"/>
       <c r="N17" s="1"/>

</xml_diff>